<commit_message>
completion of carbon measurement experiment. Updated data and analysis.
</commit_message>
<xml_diff>
--- a/data/carbon/Cadiz2025_Biomass_C_cores.xlsx
+++ b/data/carbon/Cadiz2025_Biomass_C_cores.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REWRITE\Field_data\seagrass_carbon_2025\data\carbon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REWRITE\Field_data\Nantes_cloud\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1149" uniqueCount="264">
   <si>
     <t>Core Type</t>
   </si>
@@ -897,19 +897,7 @@
     <t>Cadiz_2025_R_09</t>
   </si>
   <si>
-    <t>Cadiz_2025_R_10</t>
-  </si>
-  <si>
-    <t>Cadiz_2025_R_11</t>
-  </si>
-  <si>
     <t>Cadiz_2025_R_12</t>
-  </si>
-  <si>
-    <t>Cadiz_2025_R_13</t>
-  </si>
-  <si>
-    <t>Cadiz_2025_R_14</t>
   </si>
   <si>
     <t>Cadiz_2025_R_15</t>
@@ -956,9 +944,15 @@
     <t>spc_0</t>
   </si>
   <si>
+    <t>CarbonIC</t>
+  </si>
+  <si>
     <t>DryMassIC</t>
   </si>
   <si>
+    <t>CarbonTC</t>
+  </si>
+  <si>
     <t>DryMassTC</t>
   </si>
   <si>
@@ -977,10 +971,19 @@
     <t>bare</t>
   </si>
   <si>
-    <t>MeasuredTC</t>
-  </si>
-  <si>
-    <t>MeasuredIC</t>
+    <t>Cadiz_2025_R_10 *</t>
+  </si>
+  <si>
+    <t>Cadiz_2025_R_11 *</t>
+  </si>
+  <si>
+    <t>Cadiz_2025_R_13 *</t>
+  </si>
+  <si>
+    <t>Cadiz_2025_R_14 *</t>
+  </si>
+  <si>
+    <t>* Samples not well homogenised</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1015,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1270,7 +1273,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1347,26 +1350,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1381,6 +1366,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1661,37 +1667,37 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1702,7 +1708,7 @@
         <v>15</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>16</v>
@@ -1712,26 +1718,26 @@
         <v>Cadiz_2025_L_01</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G2" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E2, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>8460</v>
       </c>
       <c r="H2" s="6">
-        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E2,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E2&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>97.99</v>
       </c>
       <c r="I2" s="6">
-        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E2,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E2&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>31.56</v>
       </c>
       <c r="J2" s="6">
-        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E2,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E2&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>315.60000000000002</v>
       </c>
       <c r="K2" s="6">
-        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E2,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F2= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E2&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.6080000000000001</v>
       </c>
     </row>
@@ -1743,7 +1749,7 @@
         <v>15</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>18</v>
@@ -1753,26 +1759,26 @@
         <v>Cadiz_2025_L_02</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G3" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E3, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>14302.999999999998</v>
+        <v>793.99999999999989</v>
       </c>
       <c r="H3" s="6">
-        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E3,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E3&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.47</v>
       </c>
       <c r="I3" s="6">
-        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E3,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E3&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>22.05</v>
       </c>
       <c r="J3" s="6">
-        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E3,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E3&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>351.92</v>
       </c>
       <c r="K3" s="6">
-        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E3,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F3= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E3&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.5630000000000002</v>
       </c>
       <c r="N3" s="4"/>
@@ -1785,7 +1791,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>20</v>
@@ -1795,26 +1801,26 @@
         <v>Cadiz_2025_L_03</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G4" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E4, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>13930.000000000002</v>
       </c>
       <c r="H4" s="6">
-        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E4,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E4&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>79.33</v>
       </c>
       <c r="I4" s="6">
-        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E4,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E4&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>23.98</v>
       </c>
       <c r="J4" s="6">
-        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E4,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E4&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>320.35000000000002</v>
       </c>
       <c r="K4" s="6">
-        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E4,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F4= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E4&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.6360000000000001</v>
       </c>
       <c r="N4" s="4"/>
@@ -1827,7 +1833,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>22</v>
@@ -1837,26 +1843,26 @@
         <v>Cadiz_2025_L_04</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G5" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E5, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>8146.0000000000009</v>
       </c>
       <c r="H5" s="6">
-        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E5,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E5&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>73.989999999999995</v>
       </c>
       <c r="I5" s="6">
-        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E5,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E5&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>24.5</v>
       </c>
       <c r="J5" s="6">
-        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E5,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E5&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>281.98</v>
       </c>
       <c r="K5" s="6">
-        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E5,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F5= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E5&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.1829999999999998</v>
       </c>
     </row>
@@ -1868,7 +1874,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>24</v>
@@ -1878,26 +1884,26 @@
         <v>Cadiz_2025_L_05</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G6" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E6, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>13270</v>
       </c>
       <c r="H6" s="6">
-        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E6,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E6&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>74.010000000000005</v>
       </c>
       <c r="I6" s="6">
-        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E6,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E6&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>18.350000000000001</v>
       </c>
       <c r="J6" s="6">
-        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E6,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E6&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>727.36</v>
       </c>
       <c r="K6" s="6">
-        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E6,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F6= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E6&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>6.2670000000000003</v>
       </c>
     </row>
@@ -1909,7 +1915,7 @@
         <v>15</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>26</v>
@@ -1919,26 +1925,26 @@
         <v>Cadiz_2025_L_06</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G7" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E7, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>7310</v>
       </c>
       <c r="H7" s="6">
-        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E7,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E7&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>68.98</v>
       </c>
       <c r="I7" s="6">
-        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E7,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E7&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>21.48</v>
       </c>
       <c r="J7" s="6">
-        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E7,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E7&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>657</v>
       </c>
       <c r="K7" s="6">
-        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E7,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F7= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E7&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.5510000000000002</v>
       </c>
     </row>
@@ -1950,7 +1956,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>28</v>
@@ -1960,26 +1966,26 @@
         <v>Cadiz_2025_L_07</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E8, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>10270</v>
       </c>
       <c r="H8" s="6">
-        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E8,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E8&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>73.849999999999994</v>
       </c>
       <c r="I8" s="6">
-        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E8,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E8&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>22.28</v>
       </c>
       <c r="J8" s="6">
-        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E8,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E8&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>334.55</v>
       </c>
       <c r="K8" s="6">
-        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E8,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F8= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E8&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.835</v>
       </c>
     </row>
@@ -1991,7 +1997,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>30</v>
@@ -2001,26 +2007,26 @@
         <v>Cadiz_2025_L_08</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G9" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E9, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>8690</v>
       </c>
       <c r="H9" s="6">
-        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E9,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E9&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>74.849999999999994</v>
       </c>
       <c r="I9" s="6">
-        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E9,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E9&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>24.41</v>
       </c>
       <c r="J9" s="6">
-        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E9,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E9&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>260.41000000000003</v>
       </c>
       <c r="K9" s="6">
-        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E9,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F9= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E9&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.0739999999999998</v>
       </c>
     </row>
@@ -2032,7 +2038,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>32</v>
@@ -2042,26 +2048,26 @@
         <v>Cadiz_2025_L_09</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G10" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E10, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>9430</v>
       </c>
       <c r="H10" s="6">
-        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E10,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E10&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>68.45</v>
       </c>
       <c r="I10" s="6">
-        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E10,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E10&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>23.24</v>
       </c>
       <c r="J10" s="6">
-        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E10,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E10&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>292.89999999999998</v>
       </c>
       <c r="K10" s="6">
-        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E10,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F10= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E10&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.9279999999999999</v>
       </c>
     </row>
@@ -2073,7 +2079,7 @@
         <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>34</v>
@@ -2083,26 +2089,26 @@
         <v>Cadiz_2025_L_10</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G11" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E11, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>920</v>
       </c>
       <c r="H11" s="6">
-        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E11,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E11&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>72.59</v>
       </c>
       <c r="I11" s="6">
-        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E11,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E11&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>16.37</v>
       </c>
       <c r="J11" s="6">
-        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E11,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E11&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>590.16</v>
       </c>
       <c r="K11" s="6">
-        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E11,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F11= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E11&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.2939999999999996</v>
       </c>
     </row>
@@ -2114,7 +2120,7 @@
         <v>15</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>36</v>
@@ -2124,26 +2130,26 @@
         <v>Cadiz_2025_L_11</v>
       </c>
       <c r="F12" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G12" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E12, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>722</v>
       </c>
       <c r="H12" s="6">
-        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E12,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E12&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>75.22</v>
       </c>
       <c r="I12" s="6">
-        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E12,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E12&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>23.63</v>
       </c>
       <c r="J12" s="6">
-        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E12,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E12&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>349</v>
       </c>
       <c r="K12" s="6">
-        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E12,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F12= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E12&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.524</v>
       </c>
     </row>
@@ -2155,7 +2161,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>38</v>
@@ -2165,26 +2171,26 @@
         <v>Cadiz_2025_L_12</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G13" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E13, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>593.99999999999989</v>
       </c>
       <c r="H13" s="6">
-        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E13,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E13&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>76.19</v>
       </c>
       <c r="I13" s="6">
-        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E13,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E13&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>22.04</v>
       </c>
       <c r="J13" s="6">
-        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E13,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E13&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>298.7</v>
       </c>
       <c r="K13" s="6">
-        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E13,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F13= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E13&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.5750000000000002</v>
       </c>
     </row>
@@ -2196,7 +2202,7 @@
         <v>15</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>40</v>
@@ -2206,26 +2212,26 @@
         <v>Cadiz_2025_L_13</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G14" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E14, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1181</v>
       </c>
       <c r="H14" s="6">
-        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E14,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E14&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.72</v>
       </c>
       <c r="I14" s="6">
-        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E14,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E14&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>16.399999999999999</v>
       </c>
       <c r="J14" s="6">
-        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E14,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E14&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>373.3</v>
       </c>
       <c r="K14" s="6">
-        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E14,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F14= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E14&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>8.2360000000000007</v>
       </c>
     </row>
@@ -2237,7 +2243,7 @@
         <v>15</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>42</v>
@@ -2247,26 +2253,26 @@
         <v>Cadiz_2025_L_14</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G15" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E15, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1251.9999999999998</v>
       </c>
       <c r="H15" s="6">
-        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E15,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E15&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>66.72</v>
       </c>
       <c r="I15" s="6">
-        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E15,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E15&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>16.18</v>
       </c>
       <c r="J15" s="6">
-        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E15,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E15&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>339.66</v>
       </c>
       <c r="K15" s="6">
-        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E15,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F15= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E15&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>5.8449999999999998</v>
       </c>
     </row>
@@ -2278,7 +2284,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>44</v>
@@ -2288,26 +2294,26 @@
         <v>Cadiz_2025_L_15</v>
       </c>
       <c r="F16" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G16" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E16, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1392.0000000000002</v>
       </c>
       <c r="H16" s="6">
-        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E16,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E16&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>65.709999999999994</v>
       </c>
       <c r="I16" s="6">
-        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E16,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E16&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>7.91</v>
       </c>
       <c r="J16" s="6">
-        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E16,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E16&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>529.88</v>
       </c>
       <c r="K16" s="6">
-        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E16,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F16= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E16&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>8.02</v>
       </c>
     </row>
@@ -2319,7 +2325,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>46</v>
@@ -2329,26 +2335,26 @@
         <v>Cadiz_2025_L_16</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G17" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E17, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1111</v>
       </c>
       <c r="H17" s="6">
-        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E17,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E17&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>68.989999999999995</v>
       </c>
       <c r="I17" s="6">
-        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E17,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E17&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>18.23</v>
       </c>
       <c r="J17" s="6">
-        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E17,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E17&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>386.41</v>
       </c>
       <c r="K17" s="6">
-        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E17,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F17= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E17&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.0739999999999998</v>
       </c>
     </row>
@@ -2360,7 +2366,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>48</v>
@@ -2370,26 +2376,26 @@
         <v>Cadiz_2025_L_17</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G18" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E18, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1141.0000000000002</v>
       </c>
       <c r="H18" s="6">
-        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E18,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E18&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>71.47</v>
       </c>
       <c r="I18" s="6">
-        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E18,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E18&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>17.64</v>
       </c>
       <c r="J18" s="6">
-        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E18,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E18&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>393.52</v>
       </c>
       <c r="K18" s="6">
-        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E18,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F18= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E18&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.496</v>
       </c>
     </row>
@@ -2401,7 +2407,7 @@
         <v>15</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>50</v>
@@ -2411,26 +2417,26 @@
         <v>Cadiz_2025_L_18</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G19" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E19, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>-531</v>
       </c>
       <c r="H19" s="6">
-        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E19,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E19&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I19" s="6">
-        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E19,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E19&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J19" s="6">
-        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E19,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E19&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K19" s="6">
-        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E19,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F19= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E19&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2442,7 +2448,7 @@
         <v>15</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>52</v>
@@ -2452,26 +2458,26 @@
         <v>Cadiz_2025_L_19</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G20" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E20, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>50.999999999999993</v>
       </c>
       <c r="H20" s="6">
-        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E20,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E20&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I20" s="6">
-        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E20,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E20&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J20" s="6">
-        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E20,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E20&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K20" s="6">
-        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E20,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F20= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E20&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2483,7 +2489,7 @@
         <v>15</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>54</v>
@@ -2493,26 +2499,26 @@
         <v>Cadiz_2025_L_20</v>
       </c>
       <c r="F21" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G21" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E21, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H21" s="6">
-        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E21,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E21&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I21" s="6">
-        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E21,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E21&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J21" s="6">
-        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E21,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E21&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K21" s="6">
-        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E21,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F21= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E21&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2524,7 +2530,7 @@
         <v>15</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>57</v>
@@ -2534,26 +2540,26 @@
         <v>Cadiz_2025_L_21</v>
       </c>
       <c r="F22" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G22" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E22, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>22.000000000000021</v>
       </c>
       <c r="H22" s="6">
-        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E22,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E22&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I22" s="6">
-        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E22,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E22&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J22" s="6">
-        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E22,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E22&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K22" s="6">
-        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E22,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F22= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E22&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2565,7 +2571,7 @@
         <v>15</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>59</v>
@@ -2575,26 +2581,26 @@
         <v>Cadiz_2025_L_22</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G23" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E23, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>1444</v>
       </c>
       <c r="H23" s="6">
-        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E23,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E23&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I23" s="6">
-        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E23,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E23&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J23" s="6">
-        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E23,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E23&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K23" s="6">
-        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E23,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F23= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E23&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2606,7 +2612,7 @@
         <v>15</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>61</v>
@@ -2616,26 +2622,26 @@
         <v>Cadiz_2025_L_23</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G24" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E24, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H24" s="6">
-        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E24,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E24&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I24" s="6">
-        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E24,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E24&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J24" s="6">
-        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E24,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E24&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K24" s="6">
-        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E24,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F24= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E24&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2647,7 +2653,7 @@
         <v>15</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>63</v>
@@ -2657,26 +2663,26 @@
         <v>Cadiz_2025_L_24</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G25" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E25, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>19.000000000000018</v>
       </c>
       <c r="H25" s="6">
-        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E25,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E25&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I25" s="6">
-        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E25,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E25&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J25" s="6">
-        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E25,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E25&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K25" s="6">
-        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E25,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F25= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E25&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2688,7 +2694,7 @@
         <v>15</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>65</v>
@@ -2698,26 +2704,26 @@
         <v>Cadiz_2025_L_25</v>
       </c>
       <c r="F26" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G26" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E26, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>39.000000000000036</v>
       </c>
       <c r="H26" s="6">
-        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E26,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E26&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I26" s="6">
-        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E26,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E26&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J26" s="6">
-        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E26,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E26&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K26" s="6">
-        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E26,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F26= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E26&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2729,7 +2735,7 @@
         <v>15</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>67</v>
@@ -2739,26 +2745,26 @@
         <v>Cadiz_2025_L_26</v>
       </c>
       <c r="F27" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G27" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E27, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
-        <v>0</v>
+        <v>14.000000000000012</v>
       </c>
       <c r="H27" s="6">
-        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E27,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E27&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I27" s="6">
-        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E27,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E27&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J27" s="6">
-        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E27,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E27&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K27" s="6">
-        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E27,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F27= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E27&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -2787,19 +2793,19 @@
         <v>NA</v>
       </c>
       <c r="H28" s="6" t="str">
-        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E28,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E28&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I28" s="6" t="str">
-        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E28,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E28&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J28" s="6" t="str">
-        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E28,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E28&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K28" s="6" t="str">
-        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E28,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F28= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E28&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -2828,19 +2834,19 @@
         <v>NA</v>
       </c>
       <c r="H29" s="6" t="str">
-        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E29,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E29&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I29" s="6" t="str">
-        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E29,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E29&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J29" s="6" t="str">
-        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E29,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E29&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K29" s="6" t="str">
-        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E29,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F29= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E29&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -2869,19 +2875,19 @@
         <v>NA</v>
       </c>
       <c r="H30" s="6" t="str">
-        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E30,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E30&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I30" s="6" t="str">
-        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E30,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E30&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J30" s="6" t="str">
-        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E30,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E30&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K30" s="6" t="str">
-        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E30,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F30= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E30&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -2910,19 +2916,19 @@
         <v>NA</v>
       </c>
       <c r="H31" s="6" t="str">
-        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E31,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E31&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I31" s="6" t="str">
-        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E31,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E31&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J31" s="6" t="str">
-        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E31,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E31&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K31" s="6" t="str">
-        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E31,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F31= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E31&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -2934,7 +2940,7 @@
         <v>77</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>16</v>
@@ -2944,26 +2950,26 @@
         <v>Cadiz_2025_R_01</v>
       </c>
       <c r="F32" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G32" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E32, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1648.0000000000002</v>
       </c>
       <c r="H32" s="6">
-        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E32,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E32&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.86</v>
       </c>
       <c r="I32" s="6">
-        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E32,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E32&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>22.58</v>
       </c>
       <c r="J32" s="6">
-        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E32,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E32&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>353.87</v>
       </c>
       <c r="K32" s="6">
-        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E32,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F32= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E32&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.3210000000000002</v>
       </c>
     </row>
@@ -2975,7 +2981,7 @@
         <v>77</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>18</v>
@@ -2985,26 +2991,26 @@
         <v>Cadiz_2025_R_02</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G33" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E33, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1374</v>
       </c>
       <c r="H33" s="6">
-        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E33,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E33&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>72.069999999999993</v>
       </c>
       <c r="I33" s="6">
-        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E33,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E33&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>24.34</v>
       </c>
       <c r="J33" s="6">
-        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E33,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E33&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>395</v>
       </c>
       <c r="K33" s="6">
-        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E33,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F33= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E33&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.1420000000000003</v>
       </c>
     </row>
@@ -3016,7 +3022,7 @@
         <v>77</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>20</v>
@@ -3026,26 +3032,26 @@
         <v>Cadiz_2025_R_03</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G34" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E34, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1428</v>
       </c>
       <c r="H34" s="6">
-        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E34,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E34&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.98</v>
       </c>
       <c r="I34" s="6">
-        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E34,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E34&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>20.7</v>
       </c>
       <c r="J34" s="6">
-        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E34,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E34&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>366.05</v>
       </c>
       <c r="K34" s="6">
-        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E34,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F34= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E34&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.0979999999999999</v>
       </c>
     </row>
@@ -3057,7 +3063,7 @@
         <v>77</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>22</v>
@@ -3067,26 +3073,26 @@
         <v>Cadiz_2025_R_04</v>
       </c>
       <c r="F35" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G35" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E35, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>2036</v>
       </c>
       <c r="H35" s="6">
-        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E35,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E35&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>78.81</v>
       </c>
       <c r="I35" s="6">
-        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E35,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E35&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>28.05</v>
       </c>
       <c r="J35" s="6">
-        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E35,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E35&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>363.62</v>
       </c>
       <c r="K35" s="6">
-        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E35,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F35= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E35&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.1779999999999999</v>
       </c>
     </row>
@@ -3098,7 +3104,7 @@
         <v>77</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>24</v>
@@ -3108,26 +3114,26 @@
         <v>Cadiz_2025_R_05</v>
       </c>
       <c r="F36" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G36" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E36, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1189</v>
       </c>
       <c r="H36" s="6">
-        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E36,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E36&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.709999999999994</v>
       </c>
       <c r="I36" s="6">
-        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E36,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E36&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>17.399999999999999</v>
       </c>
       <c r="J36" s="6">
-        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E36,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E36&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>341.9</v>
       </c>
       <c r="K36" s="6">
-        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E36,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F36= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E36&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.41</v>
       </c>
     </row>
@@ -3139,7 +3145,7 @@
         <v>77</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>26</v>
@@ -3149,26 +3155,26 @@
         <v>Cadiz_2025_R_06</v>
       </c>
       <c r="F37" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G37" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E37, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1815.9999999999998</v>
       </c>
       <c r="H37" s="6">
-        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E37,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E37&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>73.91</v>
       </c>
       <c r="I37" s="6">
-        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E37,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E37&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>24.79</v>
       </c>
       <c r="J37" s="6">
-        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E37,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E37&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>365.95</v>
       </c>
       <c r="K37" s="6">
-        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E37,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F37= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E37&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.41</v>
       </c>
     </row>
@@ -3180,7 +3186,7 @@
         <v>77</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>28</v>
@@ -3190,26 +3196,26 @@
         <v>Cadiz_2025_R_07</v>
       </c>
       <c r="F38" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G38" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E38, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>2762</v>
       </c>
       <c r="H38" s="6">
-        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E38,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E38&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>74.569999999999993</v>
       </c>
       <c r="I38" s="6">
-        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E38,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E38&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>23.16</v>
       </c>
       <c r="J38" s="6">
-        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E38,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E38&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>302.08</v>
       </c>
       <c r="K38" s="6">
-        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E38,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F38= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E38&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.8479999999999999</v>
       </c>
     </row>
@@ -3221,7 +3227,7 @@
         <v>77</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>30</v>
@@ -3231,26 +3237,26 @@
         <v>Cadiz_2025_R_08</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G39" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E39, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1477</v>
       </c>
       <c r="H39" s="6">
-        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E39,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E39&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>78.72</v>
       </c>
       <c r="I39" s="6">
-        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E39,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E39&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>25.66</v>
       </c>
       <c r="J39" s="6">
-        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E39,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E39&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>463.97</v>
       </c>
       <c r="K39" s="6">
-        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E39,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F39= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E39&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.4039999999999999</v>
       </c>
     </row>
@@ -3262,7 +3268,7 @@
         <v>77</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>32</v>
@@ -3272,26 +3278,26 @@
         <v>Cadiz_2025_R_09</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G40" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E40, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>3114</v>
       </c>
       <c r="H40" s="6">
-        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E40,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E40&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>72.12</v>
       </c>
       <c r="I40" s="6">
-        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E40,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E40&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>24.95</v>
       </c>
       <c r="J40" s="6">
-        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E40,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E40&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>725.53</v>
       </c>
       <c r="K40" s="6">
-        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E40,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F40= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E40&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>5.9690000000000003</v>
       </c>
     </row>
@@ -3303,7 +3309,7 @@
         <v>77</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>34</v>
@@ -3313,26 +3319,26 @@
         <v>Cadiz_2025_R_10</v>
       </c>
       <c r="F41" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G41" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E41, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1288</v>
       </c>
       <c r="H41" s="6">
-        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E41&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>76.180000000000007</v>
       </c>
       <c r="I41" s="6">
-        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E41&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>15.92</v>
       </c>
       <c r="J41" s="6">
-        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E41&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>340.23</v>
       </c>
       <c r="K41" s="6">
-        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F41= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E41&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>1.5369999999999999</v>
       </c>
     </row>
@@ -3344,7 +3350,7 @@
         <v>77</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>36</v>
@@ -3354,26 +3360,26 @@
         <v>Cadiz_2025_R_11</v>
       </c>
       <c r="F42" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G42" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E42, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>771.99999999999989</v>
       </c>
       <c r="H42" s="6">
-        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E42&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>79.510000000000005</v>
       </c>
       <c r="I42" s="6">
-        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E42&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>21.39</v>
       </c>
       <c r="J42" s="6">
-        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E42&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>485.75</v>
       </c>
       <c r="K42" s="6">
-        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F42= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E42&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>1.2010000000000001</v>
       </c>
     </row>
@@ -3385,7 +3391,7 @@
         <v>77</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>38</v>
@@ -3395,26 +3401,26 @@
         <v>Cadiz_2025_R_12</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G43" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E43, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1548</v>
       </c>
       <c r="H43" s="6">
-        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E43,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E43&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>78.709999999999994</v>
       </c>
       <c r="I43" s="6">
-        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E43,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E43&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>13.23</v>
       </c>
       <c r="J43" s="6">
-        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E43,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E43&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>344.57</v>
       </c>
       <c r="K43" s="6">
-        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E43,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F43= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E43&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.6819999999999999</v>
       </c>
     </row>
@@ -3426,7 +3432,7 @@
         <v>77</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>40</v>
@@ -3436,26 +3442,26 @@
         <v>Cadiz_2025_R_13</v>
       </c>
       <c r="F44" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G44" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E44, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1611</v>
       </c>
       <c r="H44" s="6">
-        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E44&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>71.760000000000005</v>
       </c>
       <c r="I44" s="6">
-        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E44&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>18.350000000000001</v>
       </c>
       <c r="J44" s="6">
-        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E44&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>263.48</v>
       </c>
       <c r="K44" s="6">
-        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F44= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E44&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.6760000000000002</v>
       </c>
     </row>
@@ -3467,7 +3473,7 @@
         <v>77</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>42</v>
@@ -3477,26 +3483,26 @@
         <v>Cadiz_2025_R_14</v>
       </c>
       <c r="F45" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G45" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E45, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>402.00000000000011</v>
       </c>
       <c r="H45" s="6">
-        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E45&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>72.569999999999993</v>
       </c>
       <c r="I45" s="6">
-        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E45&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>17.3</v>
       </c>
       <c r="J45" s="6">
-        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E45&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>265.94</v>
       </c>
       <c r="K45" s="6">
-        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F45= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E45&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.6</v>
       </c>
     </row>
@@ -3508,7 +3514,7 @@
         <v>77</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>44</v>
@@ -3518,26 +3524,26 @@
         <v>Cadiz_2025_R_15</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G46" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E46, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>957.00000000000011</v>
       </c>
       <c r="H46" s="6">
-        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E46,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E46&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>77.930000000000007</v>
       </c>
       <c r="I46" s="6">
-        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E46,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E46&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>9.7370000000000001</v>
       </c>
       <c r="J46" s="6">
-        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E46,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E46&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>375.58</v>
       </c>
       <c r="K46" s="6">
-        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E46,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F46= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E46&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>3.6509999999999998</v>
       </c>
     </row>
@@ -3549,7 +3555,7 @@
         <v>77</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>46</v>
@@ -3559,26 +3565,26 @@
         <v>Cadiz_2025_R_16</v>
       </c>
       <c r="F47" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G47" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E47, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1746</v>
       </c>
       <c r="H47" s="6">
-        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E47,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E47&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>70.400000000000006</v>
       </c>
       <c r="I47" s="6">
-        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E47,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E47&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>15.9</v>
       </c>
       <c r="J47" s="6">
-        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E47,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E47&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>456.31</v>
       </c>
       <c r="K47" s="6">
-        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E47,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F47= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E47&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>4.1790000000000003</v>
       </c>
     </row>
@@ -3590,7 +3596,7 @@
         <v>77</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>48</v>
@@ -3600,26 +3606,26 @@
         <v>Cadiz_2025_R_17</v>
       </c>
       <c r="F48" s="27" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G48" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E48, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>1768</v>
       </c>
       <c r="H48" s="6">
-        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E48,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E48&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>75.5</v>
       </c>
       <c r="I48" s="6">
-        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E48,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E48&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>15.92</v>
       </c>
       <c r="J48" s="6">
-        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E48,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E48&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>475.63</v>
       </c>
       <c r="K48" s="6">
-        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E48,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F48= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E48&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>2.6019999999999999</v>
       </c>
     </row>
@@ -3631,7 +3637,7 @@
         <v>77</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>50</v>
@@ -3641,26 +3647,26 @@
         <v>Cadiz_2025_R_18</v>
       </c>
       <c r="F49" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G49" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E49, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H49" s="6">
-        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E49,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E49&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I49" s="6">
-        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E49,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E49&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J49" s="6">
-        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E49,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E49&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K49" s="6">
-        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E49,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F49= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E49&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3672,7 +3678,7 @@
         <v>77</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>52</v>
@@ -3682,26 +3688,26 @@
         <v>Cadiz_2025_R_19</v>
       </c>
       <c r="F50" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G50" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E50, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H50" s="6">
-        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E50,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E50&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I50" s="6">
-        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E50,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E50&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J50" s="6">
-        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E50,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E50&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K50" s="6">
-        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E50,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F50= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E50&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3713,7 +3719,7 @@
         <v>77</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>54</v>
@@ -3723,26 +3729,26 @@
         <v>Cadiz_2025_R_20</v>
       </c>
       <c r="F51" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G51" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E51, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H51" s="6">
-        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E51,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E51&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I51" s="6">
-        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E51,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E51&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J51" s="6">
-        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E51,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E51&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K51" s="6">
-        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E51,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F51= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E51&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3754,7 +3760,7 @@
         <v>77</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>57</v>
@@ -3764,26 +3770,26 @@
         <v>Cadiz_2025_R_21</v>
       </c>
       <c r="F52" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G52" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E52, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H52" s="6">
-        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E52,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E52&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I52" s="6">
-        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E52,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E52&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J52" s="6">
-        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E52,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E52&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K52" s="6">
-        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E52,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F52= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E52&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3795,7 +3801,7 @@
         <v>77</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>59</v>
@@ -3805,26 +3811,26 @@
         <v>Cadiz_2025_R_22</v>
       </c>
       <c r="F53" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G53" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E53, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H53" s="6">
-        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E53,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E53&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I53" s="6">
-        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E53,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E53&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J53" s="6">
-        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E53,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E53&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K53" s="6">
-        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E53,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F53= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E53&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3836,7 +3842,7 @@
         <v>77</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>61</v>
@@ -3846,26 +3852,26 @@
         <v>Cadiz_2025_R_23</v>
       </c>
       <c r="F54" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G54" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E54, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H54" s="6">
-        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E54,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E54&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I54" s="6">
-        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E54,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E54&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J54" s="6">
-        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E54,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E54&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K54" s="6">
-        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E54,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F54= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E54&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3877,7 +3883,7 @@
         <v>77</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>63</v>
@@ -3887,26 +3893,26 @@
         <v>Cadiz_2025_R_24</v>
       </c>
       <c r="F55" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G55" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E55, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H55" s="6">
-        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E55,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E55&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I55" s="6">
-        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E55,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E55&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J55" s="6">
-        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E55,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E55&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K55" s="6">
-        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E55,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F55= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E55&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3918,7 +3924,7 @@
         <v>77</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>65</v>
@@ -3928,26 +3934,26 @@
         <v>Cadiz_2025_R_25</v>
       </c>
       <c r="F56" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G56" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E56, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H56" s="6">
-        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E56,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E56&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I56" s="6">
-        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E56,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E56&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J56" s="6">
-        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E56,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E56&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K56" s="6">
-        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E56,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F56= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E56&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -3959,7 +3965,7 @@
         <v>77</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>67</v>
@@ -3969,26 +3975,26 @@
         <v>Cadiz_2025_R_26</v>
       </c>
       <c r="F57" s="27" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G57" s="6">
         <f>IFERROR(VLOOKUP(CONCATENATE(E57, "_01"),raw!$E$2:$J$61,6)*1000, "NA")</f>
         <v>0</v>
       </c>
       <c r="H57" s="6">
-        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E57,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E57&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>0</v>
       </c>
       <c r="I57" s="6">
-        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E57,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E57&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>0</v>
       </c>
       <c r="J57" s="6">
-        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E57,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E57&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>0</v>
       </c>
       <c r="K57" s="6">
-        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E57,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F57= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E57&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>0</v>
       </c>
     </row>
@@ -4017,19 +4023,19 @@
         <v>NA</v>
       </c>
       <c r="H58" s="6" t="str">
-        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E58,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E58&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I58" s="6" t="str">
-        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E58,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E58&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J58" s="6" t="str">
-        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E58,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E58&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K58" s="6" t="str">
-        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E58,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F58= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E58&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -4058,19 +4064,19 @@
         <v>NA</v>
       </c>
       <c r="H59" s="6" t="str">
-        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E59,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E59&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I59" s="6" t="str">
-        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E59,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E59&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J59" s="6" t="str">
-        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E59,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E59&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K59" s="6" t="str">
-        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E59,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F59= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E59&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -4099,19 +4105,19 @@
         <v>NA</v>
       </c>
       <c r="H60" s="6" t="str">
-        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E60,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E60&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I60" s="6" t="str">
-        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E60,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E60&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J60" s="6" t="str">
-        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E60,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E60&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K60" s="6" t="str">
-        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E60,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F60= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E60&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -4140,19 +4146,19 @@
         <v>NA</v>
       </c>
       <c r="H61" s="6" t="str">
-        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E61,carbon!$A$14:$A$48,0),2), "NA") )</f>
+        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E61&amp;"*",carbon!$A$14:$A$48,0),2), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="I61" s="6" t="str">
-        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E61,carbon!$A$14:$A$48,0),4), "NA") )</f>
+        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E61&amp;"*",carbon!$A$14:$A$48,0),4), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="J61" s="6" t="str">
-        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E61,carbon!$A$14:$A$48,0),6), "NA") )</f>
+        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E61&amp;"*",carbon!$A$14:$A$48,0),6), "NA") )</f>
         <v>NA</v>
       </c>
       <c r="K61" s="6" t="str">
-        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E61,carbon!$A$14:$A$48,0),8), "NA") )</f>
+        <f>IF($F61= "bare", 0, IFERROR(INDEX(carbon!$A$14:$J$48,MATCH("*"&amp;data!$E61&amp;"*",carbon!$A$14:$A$48,0),8), "NA") )</f>
         <v>NA</v>
       </c>
     </row>
@@ -4258,7 +4264,7 @@
         <v>91.059999999999988</v>
       </c>
       <c r="J2" s="6">
-        <f>IFERROR(IF(+H2-F2 &lt; 0, 0, +H2-F2), "NA")</f>
+        <f>IFERROR(+H2-F2, "NA")</f>
         <v>8.4600000000000009</v>
       </c>
       <c r="K2" s="6">
@@ -4308,15 +4314,15 @@
         <v>93.39</v>
       </c>
       <c r="H3" s="3">
-        <v>15.01</v>
+        <v>1.5009999999999999</v>
       </c>
       <c r="I3" s="6">
         <f t="shared" si="0"/>
         <v>92.683000000000007</v>
       </c>
       <c r="J3" s="6">
-        <f t="shared" ref="J3:J61" si="1">IFERROR(IF(+H3-F3 &lt; 0, 0, +H3-F3), "NA")</f>
-        <v>14.302999999999999</v>
+        <f t="shared" ref="J3:J61" si="1">IFERROR(+H3-F3, "NA")</f>
+        <v>0.79399999999999993</v>
       </c>
       <c r="K3" s="6">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E3,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5151,7 +5157,7 @@
         <v>51</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>0.53100000000000003</v>
       </c>
       <c r="G19" s="3">
         <v>0</v>
@@ -5164,7 +5170,7 @@
       </c>
       <c r="J19" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.53100000000000003</v>
       </c>
       <c r="K19" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E19,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5200,21 +5206,21 @@
         <v>53</v>
       </c>
       <c r="F20" s="3">
-        <v>0</v>
+        <v>0.38800000000000001</v>
       </c>
       <c r="G20" s="3">
-        <v>0</v>
+        <v>0.54400000000000004</v>
       </c>
       <c r="H20" s="3">
-        <v>0</v>
+        <v>0.439</v>
       </c>
       <c r="I20" s="6">
         <f>+G20-F20</f>
-        <v>0</v>
+        <v>0.15600000000000003</v>
       </c>
       <c r="J20" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5.099999999999999E-2</v>
       </c>
       <c r="K20" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E20,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5299,21 +5305,21 @@
         <v>58</v>
       </c>
       <c r="F22" s="3">
-        <v>0</v>
+        <v>0.50800000000000001</v>
       </c>
       <c r="G22" s="3">
-        <v>0</v>
+        <v>0.59099999999999997</v>
       </c>
       <c r="H22" s="3">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="I22" s="6">
         <f t="shared" ref="I22:I48" si="2">+G22-F22</f>
-        <v>0</v>
+        <v>8.2999999999999963E-2</v>
       </c>
       <c r="J22" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.200000000000002E-2</v>
       </c>
       <c r="K22" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E22,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5349,21 +5355,21 @@
         <v>60</v>
       </c>
       <c r="F23" s="3">
-        <v>0</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="G23" s="3">
-        <v>0</v>
+        <v>16.332999999999998</v>
       </c>
       <c r="H23" s="3">
-        <v>0</v>
+        <v>1.919</v>
       </c>
       <c r="I23" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15.857999999999999</v>
       </c>
       <c r="J23" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.444</v>
       </c>
       <c r="K23" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E23,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5448,21 +5454,21 @@
         <v>64</v>
       </c>
       <c r="F25" s="3">
-        <v>0</v>
+        <v>0.46899999999999997</v>
       </c>
       <c r="G25" s="3">
-        <v>0</v>
+        <v>0.52900000000000003</v>
       </c>
       <c r="H25" s="3">
-        <v>0</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="I25" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="J25" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.9000000000000017E-2</v>
       </c>
       <c r="K25" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E25,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5498,21 +5504,21 @@
         <v>66</v>
       </c>
       <c r="F26" s="3">
-        <v>0</v>
+        <v>0.89300000000000002</v>
       </c>
       <c r="G26" s="3">
-        <v>0</v>
+        <v>1.0549999999999999</v>
       </c>
       <c r="H26" s="3">
-        <v>0</v>
+        <v>0.93200000000000005</v>
       </c>
       <c r="I26" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.16199999999999992</v>
       </c>
       <c r="J26" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.9000000000000035E-2</v>
       </c>
       <c r="K26" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E26,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5548,21 +5554,21 @@
         <v>68</v>
       </c>
       <c r="F27" s="3">
-        <v>0</v>
+        <v>0.65900000000000003</v>
       </c>
       <c r="G27" s="3">
-        <v>0</v>
+        <v>0.747</v>
       </c>
       <c r="H27" s="3">
-        <v>0</v>
+        <v>0.67300000000000004</v>
       </c>
       <c r="I27" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>8.7999999999999967E-2</v>
       </c>
       <c r="J27" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.4000000000000012E-2</v>
       </c>
       <c r="K27" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E27,carbon!$A$14:$A$48,0),2), "NA")</f>
@@ -5610,23 +5616,23 @@
         <v>56</v>
       </c>
       <c r="J28" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J28" si="3">IFERROR(+H28-F28, "NA")</f>
         <v>NA</v>
       </c>
       <c r="K28" s="6" t="str">
-        <f t="shared" ref="K28" si="3">IFERROR(+I28-G28, "NA")</f>
+        <f t="shared" ref="K28" si="4">IFERROR(+I28-G28, "NA")</f>
         <v>NA</v>
       </c>
       <c r="L28" s="6" t="str">
-        <f t="shared" ref="L28" si="4">IFERROR(+J28-H28, "NA")</f>
+        <f t="shared" ref="L28" si="5">IFERROR(+J28-H28, "NA")</f>
         <v>NA</v>
       </c>
       <c r="M28" s="6" t="str">
-        <f t="shared" ref="M28" si="5">IFERROR(+K28-I28, "NA")</f>
+        <f t="shared" ref="M28" si="6">IFERROR(+K28-I28, "NA")</f>
         <v>NA</v>
       </c>
       <c r="N28" s="6" t="str">
-        <f t="shared" ref="N28" si="6">IFERROR(+L28-J28, "NA")</f>
+        <f t="shared" ref="N28" si="7">IFERROR(+L28-J28, "NA")</f>
         <v>NA</v>
       </c>
     </row>
@@ -5663,19 +5669,19 @@
         <v>NA</v>
       </c>
       <c r="K29" s="6" t="str">
-        <f t="shared" ref="K29:K31" si="7">IFERROR(+I29-G29, "NA")</f>
+        <f t="shared" ref="K29:K31" si="8">IFERROR(+I29-G29, "NA")</f>
         <v>NA</v>
       </c>
       <c r="L29" s="6" t="str">
-        <f t="shared" ref="L29:L31" si="8">IFERROR(+J29-H29, "NA")</f>
+        <f t="shared" ref="L29:L31" si="9">IFERROR(+J29-H29, "NA")</f>
         <v>NA</v>
       </c>
       <c r="M29" s="6" t="str">
-        <f t="shared" ref="M29:M31" si="9">IFERROR(+K29-I29, "NA")</f>
+        <f t="shared" ref="M29:M31" si="10">IFERROR(+K29-I29, "NA")</f>
         <v>NA</v>
       </c>
       <c r="N29" s="6" t="str">
-        <f t="shared" ref="N29:N31" si="10">IFERROR(+L29-J29, "NA")</f>
+        <f t="shared" ref="N29:N31" si="11">IFERROR(+L29-J29, "NA")</f>
         <v>NA</v>
       </c>
     </row>
@@ -5712,19 +5718,19 @@
         <v>NA</v>
       </c>
       <c r="K30" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>NA</v>
       </c>
       <c r="L30" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>NA</v>
       </c>
       <c r="M30" s="6" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>NA</v>
       </c>
       <c r="N30" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>NA</v>
       </c>
     </row>
@@ -5761,19 +5767,19 @@
         <v>NA</v>
       </c>
       <c r="K31" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>NA</v>
       </c>
       <c r="L31" s="6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>NA</v>
       </c>
       <c r="M31" s="6" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>NA</v>
       </c>
       <c r="N31" s="6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>NA</v>
       </c>
     </row>
@@ -6260,21 +6266,21 @@
         <f t="shared" si="1"/>
         <v>1.288</v>
       </c>
-      <c r="K41" s="6">
+      <c r="K41" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),2), "NA")</f>
-        <v>76.180000000000007</v>
-      </c>
-      <c r="L41" s="6">
+        <v>NA</v>
+      </c>
+      <c r="L41" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),4), "NA")</f>
-        <v>15.92</v>
-      </c>
-      <c r="M41" s="6">
+        <v>NA</v>
+      </c>
+      <c r="M41" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),6), "NA")</f>
-        <v>340.23</v>
-      </c>
-      <c r="N41" s="6">
+        <v>NA</v>
+      </c>
+      <c r="N41" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E41,carbon!$A$14:$A$48,0),8), "NA")</f>
-        <v>1.5369999999999999</v>
+        <v>NA</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="15">
@@ -6310,21 +6316,21 @@
         <f t="shared" si="1"/>
         <v>0.77199999999999991</v>
       </c>
-      <c r="K42" s="6">
+      <c r="K42" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),2), "NA")</f>
-        <v>79.510000000000005</v>
-      </c>
-      <c r="L42" s="6">
+        <v>NA</v>
+      </c>
+      <c r="L42" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),4), "NA")</f>
-        <v>21.39</v>
-      </c>
-      <c r="M42" s="6">
+        <v>NA</v>
+      </c>
+      <c r="M42" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),6), "NA")</f>
-        <v>485.75</v>
-      </c>
-      <c r="N42" s="6">
+        <v>NA</v>
+      </c>
+      <c r="N42" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E42,carbon!$A$14:$A$48,0),8), "NA")</f>
-        <v>1.2010000000000001</v>
+        <v>NA</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="15">
@@ -6410,21 +6416,21 @@
         <f t="shared" si="1"/>
         <v>1.611</v>
       </c>
-      <c r="K44" s="6">
+      <c r="K44" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),2), "NA")</f>
-        <v>71.760000000000005</v>
-      </c>
-      <c r="L44" s="6">
+        <v>NA</v>
+      </c>
+      <c r="L44" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),4), "NA")</f>
-        <v>18.350000000000001</v>
-      </c>
-      <c r="M44" s="6">
+        <v>NA</v>
+      </c>
+      <c r="M44" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),6), "NA")</f>
-        <v>263.48</v>
-      </c>
-      <c r="N44" s="6">
+        <v>NA</v>
+      </c>
+      <c r="N44" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E44,carbon!$A$14:$A$48,0),8), "NA")</f>
-        <v>2.6760000000000002</v>
+        <v>NA</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="15">
@@ -6460,21 +6466,21 @@
         <f t="shared" si="1"/>
         <v>0.40200000000000014</v>
       </c>
-      <c r="K45" s="6">
+      <c r="K45" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),2), "NA")</f>
-        <v>72.569999999999993</v>
-      </c>
-      <c r="L45" s="6">
+        <v>NA</v>
+      </c>
+      <c r="L45" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),4), "NA")</f>
-        <v>17.3</v>
-      </c>
-      <c r="M45" s="6">
+        <v>NA</v>
+      </c>
+      <c r="M45" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),6), "NA")</f>
-        <v>265.94</v>
-      </c>
-      <c r="N45" s="6">
+        <v>NA</v>
+      </c>
+      <c r="N45" s="6" t="str">
         <f>IFERROR(INDEX(carbon!$A$14:$J$48,MATCH(data!$E45,carbon!$A$14:$A$48,0),8), "NA")</f>
-        <v>2.6</v>
+        <v>NA</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="15">
@@ -7097,23 +7103,23 @@
         <v>56</v>
       </c>
       <c r="J58" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J58" si="12">IFERROR(+H58-F58, "NA")</f>
         <v>NA</v>
       </c>
       <c r="K58" s="6" t="str">
-        <f t="shared" ref="K58" si="11">IFERROR(+I58-G58, "NA")</f>
+        <f t="shared" ref="K58" si="13">IFERROR(+I58-G58, "NA")</f>
         <v>NA</v>
       </c>
       <c r="L58" s="6" t="str">
-        <f t="shared" ref="L58" si="12">IFERROR(+J58-H58, "NA")</f>
+        <f t="shared" ref="L58" si="14">IFERROR(+J58-H58, "NA")</f>
         <v>NA</v>
       </c>
       <c r="M58" s="6" t="str">
-        <f t="shared" ref="M58" si="13">IFERROR(+K58-I58, "NA")</f>
+        <f t="shared" ref="M58" si="15">IFERROR(+K58-I58, "NA")</f>
         <v>NA</v>
       </c>
       <c r="N58" s="6" t="str">
-        <f t="shared" ref="N58" si="14">IFERROR(+L58-J58, "NA")</f>
+        <f t="shared" ref="N58" si="16">IFERROR(+L58-J58, "NA")</f>
         <v>NA</v>
       </c>
     </row>
@@ -7150,19 +7156,19 @@
         <v>NA</v>
       </c>
       <c r="K59" s="6" t="str">
-        <f t="shared" ref="K59:K61" si="15">IFERROR(+I59-G59, "NA")</f>
+        <f t="shared" ref="K59:K61" si="17">IFERROR(+I59-G59, "NA")</f>
         <v>NA</v>
       </c>
       <c r="L59" s="6" t="str">
-        <f t="shared" ref="L59:L61" si="16">IFERROR(+J59-H59, "NA")</f>
+        <f t="shared" ref="L59:L61" si="18">IFERROR(+J59-H59, "NA")</f>
         <v>NA</v>
       </c>
       <c r="M59" s="6" t="str">
-        <f t="shared" ref="M59:M61" si="17">IFERROR(+K59-I59, "NA")</f>
+        <f t="shared" ref="M59:M61" si="19">IFERROR(+K59-I59, "NA")</f>
         <v>NA</v>
       </c>
       <c r="N59" s="6" t="str">
-        <f t="shared" ref="N59:N61" si="18">IFERROR(+L59-J59, "NA")</f>
+        <f t="shared" ref="N59:N61" si="20">IFERROR(+L59-J59, "NA")</f>
         <v>NA</v>
       </c>
     </row>
@@ -7199,19 +7205,19 @@
         <v>NA</v>
       </c>
       <c r="K60" s="6" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>NA</v>
       </c>
       <c r="L60" s="6" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>NA</v>
       </c>
       <c r="M60" s="6" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>NA</v>
       </c>
       <c r="N60" s="6" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>NA</v>
       </c>
     </row>
@@ -7248,19 +7254,19 @@
         <v>NA</v>
       </c>
       <c r="K61" s="6" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>NA</v>
       </c>
       <c r="L61" s="6" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>NA</v>
       </c>
       <c r="M61" s="6" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>NA</v>
       </c>
       <c r="N61" s="6" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>NA</v>
       </c>
     </row>
@@ -8752,7 +8758,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="4" width="12.44140625" style="8" customWidth="1"/>
@@ -8763,78 +8769,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="28"/>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="29" t="s">
+      <c r="A1" s="38"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
       <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29" t="s">
+      <c r="A2" s="38"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
       <c r="J2" s="7"/>
     </row>
     <row r="3" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A3" s="28"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="30" t="s">
+      <c r="A3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
       <c r="J3" s="7"/>
     </row>
     <row r="5" spans="1:10" ht="18" customHeight="1">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
     </row>
     <row r="6" spans="1:10" ht="18" customHeight="1">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="34" t="s">
         <v>199</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
     </row>
     <row r="7" spans="1:10" ht="18" customHeight="1">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="1:10" ht="19.5" customHeight="1">
       <c r="A9" s="9"/>
@@ -8847,62 +8853,62 @@
     </row>
     <row r="10" spans="1:10" ht="19.5" customHeight="1">
       <c r="A10" s="10"/>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="30" t="s">
         <v>202</v>
       </c>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30" t="s">
         <v>203</v>
       </c>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
     </row>
     <row r="11" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="B11" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="C11" s="35" t="s">
+      <c r="B11" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="C11" s="29" t="s">
         <v>206</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="33" t="s">
         <v>207</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="29" t="s">
         <v>208</v>
       </c>
-      <c r="F11" s="39" t="s">
+      <c r="F11" s="33" t="s">
         <v>205</v>
       </c>
-      <c r="G11" s="35" t="s">
+      <c r="G11" s="29" t="s">
         <v>206</v>
       </c>
-      <c r="H11" s="35" t="s">
+      <c r="H11" s="29" t="s">
         <v>209</v>
       </c>
-      <c r="I11" s="35" t="s">
+      <c r="I11" s="29" t="s">
         <v>210</v>
       </c>
-      <c r="J11" s="35" t="s">
+      <c r="J11" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10" ht="14.25" customHeight="1">
       <c r="A13" s="11"/>
@@ -9846,7 +9852,7 @@
     </row>
     <row r="41" spans="1:10" ht="14.25" customHeight="1">
       <c r="A41" s="19" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="B41" s="20">
         <v>76.180000000000007</v>
@@ -9881,7 +9887,7 @@
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1">
       <c r="A42" s="19" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="B42" s="20">
         <v>79.510000000000005</v>
@@ -9916,7 +9922,7 @@
     </row>
     <row r="43" spans="1:10" ht="14.25" customHeight="1">
       <c r="A43" s="19" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B43" s="20">
         <v>78.709999999999994</v>
@@ -9951,7 +9957,7 @@
     </row>
     <row r="44" spans="1:10" ht="14.25" customHeight="1">
       <c r="A44" s="19" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="B44" s="20">
         <v>71.760000000000005</v>
@@ -9986,7 +9992,7 @@
     </row>
     <row r="45" spans="1:10" ht="14.25" customHeight="1">
       <c r="A45" s="19" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="B45" s="20">
         <v>72.569999999999993</v>
@@ -10021,7 +10027,7 @@
     </row>
     <row r="46" spans="1:10" ht="14.25" customHeight="1">
       <c r="A46" s="19" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B46" s="20">
         <v>77.930000000000007</v>
@@ -10056,7 +10062,7 @@
     </row>
     <row r="47" spans="1:10" ht="14.25" customHeight="1">
       <c r="A47" s="19" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B47" s="20">
         <v>70.400000000000006</v>
@@ -10091,7 +10097,7 @@
     </row>
     <row r="48" spans="1:10" ht="14.25" customHeight="1">
       <c r="A48" s="19" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B48" s="20">
         <v>75.5</v>
@@ -10136,8 +10142,25 @@
       <c r="I49" s="26"/>
       <c r="J49" s="23"/>
     </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="28" t="s">
+        <v>263</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:C3"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
     <mergeCell ref="I11:I12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="B10:E10"/>
@@ -10150,18 +10173,6 @@
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
     <mergeCell ref="H11:H12"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A1:C3"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.23611111111111099" right="0.23611111111111099" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="81" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>